<commit_message>
Add Brand/Login page objects and test cases, update ExtentTestManager
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/data-eCommerceCMS.xlsx
+++ b/src/test/resources/testData/data-eCommerceCMS.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22527"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SeleniumJava\FinalProject\src\test\resources\testData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Testing\Template\template\src\test\resources\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0371775-FF65-45CE-AE81-11F1EECAE0C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22A3C083-DC30-444D-AFAB-F553B54C40E3}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="2" xr2:uid="{A4C1A725-F1B3-4797-994D-1D129BC88B09}"/>
+    <workbookView xWindow="35851" yWindow="-2554" windowWidth="26083" windowHeight="13829" activeTab="2" xr2:uid="{A4C1A725-F1B3-4797-994D-1D129BC88B09}"/>
   </bookViews>
   <sheets>
     <sheet name="CategoryData" sheetId="1" r:id="rId1"/>
@@ -25,10 +25,7 @@
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -36,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="121">
   <si>
     <t>Field name</t>
   </si>
@@ -263,9 +260,6 @@
     <t>Search Logo</t>
   </si>
   <si>
-    <t>Brand 05-2024</t>
-  </si>
-  <si>
     <t>Verify</t>
   </si>
   <si>
@@ -296,9 +290,6 @@
     <t>HTML5 Brand name</t>
   </si>
   <si>
-    <t>BrandTest 05-2024</t>
-  </si>
-  <si>
     <t>search Brand</t>
   </si>
   <si>
@@ -372,6 +363,39 @@
   </si>
   <si>
     <t>Product test 5/2024</t>
+  </si>
+  <si>
+    <t>Cosy</t>
+  </si>
+  <si>
+    <t>Brand test 001</t>
+  </si>
+  <si>
+    <t>Brand test 002 edit</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Information edit (3)</t>
+  </si>
+  <si>
+    <t>Brand has been updated successfully</t>
+  </si>
+  <si>
+    <t>message edit success</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test Meta Title 123 </t>
+  </si>
+  <si>
+    <t>Test Meta des  12323</t>
+  </si>
+  <si>
+    <t>Brand Final 05-2026 02</t>
+  </si>
+  <si>
+    <t>BrandTest 05-2026</t>
+  </si>
+  <si>
+    <t>Brand 05-2026</t>
   </si>
 </sst>
 </file>
@@ -1000,19 +1024,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E40C0B0-F63E-4EAF-8795-C365E9CBE11D}">
   <dimension ref="A1:G11"/>
-  <sheetFormatPr defaultRowHeight="16.8" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="17" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" style="3"/>
-    <col min="2" max="2" width="23.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="31.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.88671875" style="1"/>
-    <col min="5" max="5" width="8.88671875" style="3"/>
-    <col min="6" max="6" width="29.6640625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="40.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="8.88671875" style="1"/>
+    <col min="1" max="1" width="8.875" style="3"/>
+    <col min="2" max="2" width="23.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.875" style="1"/>
+    <col min="5" max="5" width="8.875" style="3"/>
+    <col min="6" max="6" width="29.625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="40.875" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="8.875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="13" customFormat="1" ht="18" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" s="13" customFormat="1" ht="18.350000000000001" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>44</v>
       </c>
@@ -1040,7 +1064,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="E2" s="15">
         <v>1</v>
@@ -1092,7 +1116,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" ht="17.7" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="4">
         <v>4</v>
       </c>
@@ -1164,18 +1188,18 @@
         <v>57</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="17.7" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="7">
         <v>10</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C11" s="21" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -1187,19 +1211,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A864311-7997-448F-8B4A-34A9E676FC10}">
   <dimension ref="A1:G26"/>
-  <sheetFormatPr defaultRowHeight="16.8" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="17" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" style="1"/>
-    <col min="2" max="2" width="30.6640625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="46.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.88671875" style="1"/>
-    <col min="5" max="5" width="8.88671875" style="3"/>
-    <col min="6" max="6" width="34.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="45.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="8.88671875" style="1"/>
+    <col min="1" max="1" width="8.875" style="1"/>
+    <col min="2" max="2" width="30.625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="46.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.875" style="1"/>
+    <col min="5" max="5" width="8.875" style="3"/>
+    <col min="6" max="6" width="34.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="45.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="8.875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" ht="17.7" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="22" t="s">
         <v>59</v>
       </c>
@@ -1213,7 +1237,7 @@
         <v>59</v>
       </c>
       <c r="F1" s="26" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G1" s="24" t="s">
         <v>62</v>
@@ -1243,7 +1267,7 @@
         <v>8</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="E3" s="15">
         <v>2</v>
@@ -1263,7 +1287,7 @@
         <v>9</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="E4" s="15">
         <v>3</v>
@@ -1283,7 +1307,7 @@
         <v>10</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="E5" s="15">
         <v>4</v>
@@ -1303,7 +1327,7 @@
         <v>11</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="E6" s="15">
         <v>5</v>
@@ -1320,10 +1344,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="E7" s="15">
         <v>6</v>
@@ -1343,19 +1367,19 @@
         <v>12</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="E8" s="15">
         <v>7</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="G8" s="27" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="17.7" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="4">
         <v>8</v>
       </c>
@@ -1372,7 +1396,7 @@
         <v>20</v>
       </c>
       <c r="G9" s="9" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
@@ -1428,10 +1452,10 @@
         <v>14</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
@@ -1442,7 +1466,7 @@
         <v>17</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
@@ -1486,7 +1510,7 @@
         <v>20</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
@@ -1497,7 +1521,7 @@
         <v>21</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
@@ -1529,15 +1553,15 @@
         <v>34</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:3" ht="17.7" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="16">
         <v>24</v>
       </c>
       <c r="B25" s="19" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C25" s="21" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
@@ -1557,20 +1581,20 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59A0E0EC-1463-4A39-BDFE-97D83C26E760}">
-  <dimension ref="A1:G7"/>
-  <sheetFormatPr defaultRowHeight="16.8" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:G8"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="17" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" style="3"/>
-    <col min="2" max="2" width="23.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="31.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.88671875" style="1"/>
-    <col min="5" max="5" width="8.88671875" style="3"/>
-    <col min="6" max="6" width="29.6640625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="40.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="8.88671875" style="1"/>
+    <col min="1" max="1" width="8.875" style="3"/>
+    <col min="2" max="2" width="23.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="33.625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="8.875" style="3"/>
+    <col min="6" max="6" width="29.625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="40.875" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="8.875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="13" customFormat="1" ht="18" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" s="13" customFormat="1" ht="18.350000000000001" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>59</v>
       </c>
@@ -1578,16 +1602,19 @@
         <v>50</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>77</v>
+        <v>76</v>
+      </c>
+      <c r="D1" s="12" t="s">
+        <v>113</v>
       </c>
       <c r="E1" s="14" t="s">
         <v>59</v>
       </c>
       <c r="F1" s="17" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G1" s="12" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
@@ -1598,16 +1625,19 @@
         <v>1</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>108</v>
+        <v>111</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>112</v>
       </c>
       <c r="E2" s="15">
         <v>1</v>
       </c>
       <c r="F2" s="18" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
@@ -1618,16 +1648,19 @@
         <v>74</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>40</v>
+        <v>110</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>110</v>
       </c>
       <c r="E3" s="15">
         <v>2</v>
       </c>
       <c r="F3" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="G3" s="5" t="s">
         <v>79</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
@@ -1638,16 +1671,19 @@
         <v>3</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>86</v>
+        <v>116</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>119</v>
       </c>
       <c r="E4" s="15">
         <v>3</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
@@ -1658,47 +1694,64 @@
         <v>4</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>75</v>
+        <v>117</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>120</v>
       </c>
       <c r="E5" s="15">
         <v>4</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G5" s="20" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" ht="17.7" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="16">
         <v>5</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>108</v>
+        <v>118</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>118</v>
       </c>
       <c r="E6" s="15">
         <v>5</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="17.399999999999999" thickBot="1" x14ac:dyDescent="0.35">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="17.7" thickBot="1" x14ac:dyDescent="0.35">
       <c r="E7" s="16">
         <v>6</v>
       </c>
       <c r="F7" s="19" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="G7" s="9" t="s">
-        <v>90</v>
+        <v>88</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="17.7" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E8" s="16">
+        <v>7</v>
+      </c>
+      <c r="F8" s="19" t="s">
+        <v>115</v>
+      </c>
+      <c r="G8" s="9" t="s">
+        <v>114</v>
       </c>
     </row>
   </sheetData>

</xml_diff>